<commit_message>
Add a worked example sheet to the coder workbook
A coder who has never done this needs to see one paper already coded far more
than another paragraph of instructions. The example is Richmond p.714, where
the authors tagged the elements in their own sentence, so it shows the target
without anyone inventing one: four rows, one CMOC, with the Response-vs-Outcome
distinction spelled out underneath because that is the one both the machine and
new coders get wrong.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/gold/per_paper_coding_coder_A.xlsx
+++ b/outputs/gold/per_paper_coding_coder_A.xlsx
@@ -10,34 +10,35 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E-code reference" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="R-code reference" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S001" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S002" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S003" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S004" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S005" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S006" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S007" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S008" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S009" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S010" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S011" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S012" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S013" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S014" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S015" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S016" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S017" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S018" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S019" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S020" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S021" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S022" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S023" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S024" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S025" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S026" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S027" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S028" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EXAMPLE — read this first" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S001" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S002" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S003" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S004" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S005" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S006" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S007" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S008" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S009" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S010" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S011" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S012" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S013" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S014" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S015" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S016" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S017" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S018" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S019" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S020" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S021" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S022" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S023" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S024" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S025" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S026" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S027" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S028" sheetId="32" state="visible" r:id="rId32"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -96,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -109,6 +110,10 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -578,9 +583,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S007 (2010): Integrated Cases Section: A Course Designed to Promote Clinical Reasoning in Year 2 Medical Students</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S006 (2008): Fostering diagnostic knowledge through computer‐supported, case‐based worked examples: effects of erroneous examples and feedback</t>
         </is>
       </c>
     </row>
@@ -692,9 +697,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S008 (2010): To Think Is Good: Querying an Initial Hypothesis Reduces Diagnostic Error in Medical Students</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S007 (2010): Integrated Cases Section: A Course Designed to Promote Clinical Reasoning in Year 2 Medical Students</t>
         </is>
       </c>
     </row>
@@ -806,9 +811,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S009 (2011): A Novel Educational Tool for Teaching Diagnostic Reasoning and Laboratory Data Interpretation to Veterinary (and Medical) Students</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S008 (2010): To Think Is Good: Querying an Initial Hypothesis Reduces Diagnostic Error in Medical Students</t>
         </is>
       </c>
     </row>
@@ -920,9 +925,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S010 (2011): Bringing Explicit Insight into Cognitive Psychology Features during Clinical Reasoning Seminars: A Prospective, Controlled Study</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S009 (2011): A Novel Educational Tool for Teaching Diagnostic Reasoning and Laboratory Data Interpretation to Veterinary (and Medical) Students</t>
         </is>
       </c>
     </row>
@@ -1034,9 +1039,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S011 (2011): How we created virtual patient cases for primary care-based learning</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S010 (2011): Bringing Explicit Insight into Cognitive Psychology Features during Clinical Reasoning Seminars: A Prospective, Controlled Study</t>
         </is>
       </c>
     </row>
@@ -1148,9 +1153,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S012 (2011): The Efficacy of a Targeted Remediation Process for Students Who Fail Standardized Patient Examinations</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S011 (2011): How we created virtual patient cases for primary care-based learning</t>
         </is>
       </c>
     </row>
@@ -1262,9 +1267,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S013 (2011): The influence of medical students selfexplanations on diagnostic performance</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S012 (2011): The Efficacy of a Targeted Remediation Process for Students Who Fail Standardized Patient Examinations</t>
         </is>
       </c>
     </row>
@@ -1376,9 +1381,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S014 (2012): evPaeds: undergraduate clinical reasoning</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S013 (2011): The influence of medical students selfexplanations on diagnostic performance</t>
         </is>
       </c>
     </row>
@@ -1490,9 +1495,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S015 (2012): Preparing medical students for clinical decision making: A pilot study exploring how students make decisions and the perceived impact of a clinical decision making teaching intervention</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S014 (2012): evPaeds: undergraduate clinical reasoning</t>
         </is>
       </c>
     </row>
@@ -1604,9 +1609,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S016 (2012): Reflection as a strategy to foster medical students acquisition of diagnostic competence</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S015 (2012): Preparing medical students for clinical decision making: A pilot study exploring how students make decisions and the perceived impact of a clinical decision making teaching intervention</t>
         </is>
       </c>
     </row>
@@ -2794,9 +2799,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S017 (2012): Should we teach using schemas? Evidence from a randomised trial</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S016 (2012): Reflection as a strategy to foster medical students acquisition of diagnostic competence</t>
         </is>
       </c>
     </row>
@@ -2908,9 +2913,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S018 (2012): What and how advanced medical students learn</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S017 (2012): Should we teach using schemas? Evidence from a randomised trial</t>
         </is>
       </c>
     </row>
@@ -3022,9 +3027,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S019 (2013): Effect of enhanced analytic reasoning on diagnostic accuracy: A randomized controlled study</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S018 (2012): What and how advanced medical students learn</t>
         </is>
       </c>
     </row>
@@ -3136,9 +3141,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S020 (2013): Students selfexplanations while solving unfamiliar cases: the role of biomedical knowledge</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S019 (2013): Effect of enhanced analytic reasoning on diagnostic accuracy: A randomized controlled study</t>
         </is>
       </c>
     </row>
@@ -3250,9 +3255,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S021 (2013): To what extent does nonanalytic reasoning contribute to visual learning in cytopathology?</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S020 (2013): Students selfexplanations while solving unfamiliar cases: the role of biomedical knowledge</t>
         </is>
       </c>
     </row>
@@ -3364,9 +3369,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S022 (2014): A Serious Game Can Be a Valid Method to Train Clinical</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S021 (2013): To what extent does nonanalytic reasoning contribute to visual learning in cytopathology?</t>
         </is>
       </c>
     </row>
@@ -3478,9 +3483,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S023 (2014): Casebook: a virtual patient iPad application for teaching decision-making through the use of electronic health records</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S022 (2014): A Serious Game Can Be a Valid Method to Train Clinical</t>
         </is>
       </c>
     </row>
@@ -3592,9 +3597,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S024 (2014): Ineffectiveness of cognitive forcing strategies</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S023 (2014): Casebook: a virtual patient iPad application for teaching decision-making through the use of electronic health records</t>
         </is>
       </c>
     </row>
@@ -3706,9 +3711,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S025 (2015): Does medical students’ diagnostic performance improve by observing examples of self-explanation provided by peers or experts?</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S024 (2014): Ineffectiveness of cognitive forcing strategies</t>
         </is>
       </c>
     </row>
@@ -3820,9 +3825,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S026 (2015): Self&amp;#x2010;explanation in learning clinical reasoning: the added value of examples and prompts</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S025 (2015): Does medical students’ diagnostic performance improve by observing examples of self-explanation provided by peers or experts?</t>
         </is>
       </c>
     </row>
@@ -4856,9 +4861,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S027 (2016): Test&amp;#x2010;enhanced learning of clinical reasoning: a crossover randomised trial</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S026 (2015): Self&amp;#x2010;explanation in learning clinical reasoning: the added value of examples and prompts</t>
         </is>
       </c>
     </row>
@@ -4970,9 +4975,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S028 (None): 18  Reprinted from Australian Family Physician Vol. 41, No. 1/2 january/february 2012</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S027 (2016): Test&amp;#x2010;enhanced learning of clinical reasoning: a crossover randomised trial</t>
         </is>
       </c>
     </row>
@@ -5065,7 +5070,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5084,9 +5089,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S001 (2001): Coordination of Analytic and Similarity-Based Processing Strategies and Expertise in Dermatological Diagnosis</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S028 (None): 18  Reprinted from Australian Family Physician Vol. 41, No. 1/2 january/february 2012</t>
         </is>
       </c>
     </row>
@@ -5179,6 +5184,286 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>WORKED EXAMPLE. This is what ONE coded paper looks like. Do not edit this sheet — it is here to show you the target. Each study sheet has these same seven columns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="60" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>The source sentence is Richmond et al. (2020) p.714, where the authors marked the elements themselves:  "When an expert's reasoning processes or thoughts are explicitly revealed and discussed (Mresource) with students with sufficient domain-specific knowledge (C), this promotes understanding (Mresponse) leading to insight (Mresponse) into the reasoning process (O) and a positive learning experience (O)."   That one sentence becomes the four rows below: one CMOC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>CMOC #</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Element type</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>E-code</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Your label</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Verbatim quote</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Polarity</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Context</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>students with high domain-specific knowledge</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>students with sufficient domain-specific knowledge</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>714</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Mechanism_Resource</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>E07</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>expert's reasoning made explicit and discussed</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>an expert's reasoning processes or thoughts are explicitly revealed and discussed</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>714</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Mechanism_Response</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>E20</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>understanding of the reasoning process</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>this promotes understanding</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>714</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Outcome</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>E22</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>positive learning experience</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>a positive learning experience</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>714</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>HOW TO READ IT:</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  * All four rows share CMOC # = 1, because they are one causal story. The next story in the same paper would be CMOC # 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  * 'Your label' is your own short wording. 'Verbatim quote' must be copied from the paper exactly — if you cannot find a sentence, do not code that element.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  * E-code is the closest match from the 'E-code reference' sheet, or type NEW if the paper says something genuinely outside that list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  * Most papers give 2-5 CMOCs. Twenty means you are coding sentences, not claims.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>THE DISTINCTION PEOPLE GET WRONG MOST OFTEN:</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Mechanism_Response = inside one learner's head (understood, panicked, felt at ease).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Outcome            = a result you could put in a results table (accuracy rose, scores unchanged, similar decision speed across groups).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  'The two groups showed similar decision speed' is an OUTCOME, not a response — even though it is about learners.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -5198,9 +5483,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S002 (2003): “Clinical Reasoning Theater”</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S001 (2001): Coordination of Analytic and Similarity-Based Processing Strategies and Expertise in Dermatological Diagnosis</t>
         </is>
       </c>
     </row>
@@ -5312,9 +5597,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S003 (2006): Giving Learners the Best of Both Worlds: Do Clinical Teachers Need to Guard Against Teaching Pattern Recognition to Novices?</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S002 (2003): “Clinical Reasoning Theater”</t>
         </is>
       </c>
     </row>
@@ -5426,9 +5711,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S004 (2007): Teaching from the clinical reasoning literature: combined reasoning strategies help novice diagnosticians overcome misleading information</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S003 (2006): Giving Learners the Best of Both Worlds: Do Clinical Teachers Need to Guard Against Teaching Pattern Recognition to Novices?</t>
         </is>
       </c>
     </row>
@@ -5540,9 +5825,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S005 (2007): The benefits of flexibility: the pedagogical value of instructions to adopt multifaceted diagnostic reasoning strategies</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S004 (2007): Teaching from the clinical reasoning literature: combined reasoning strategies help novice diagnosticians overcome misleading information</t>
         </is>
       </c>
     </row>
@@ -5654,9 +5939,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>S006 (2008): Fostering diagnostic knowledge through computer‐supported, case‐based worked examples: effects of erroneous examples and feedback</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>S005 (2007): The benefits of flexibility: the pedagogical value of instructions to adopt multifaceted diagnostic reasoning strategies</t>
         </is>
       </c>
     </row>

</xml_diff>